<commit_message>
Remove hardcoded Golden checks from verification output; fix Arrow serialization by using numeric thresholds
</commit_message>
<xml_diff>
--- a/output/report.xlsx
+++ b/output/report.xlsx
@@ -884,8 +884,8 @@
     <col width="9" customWidth="1" min="16" max="16"/>
     <col width="18" customWidth="1" min="17" max="17"/>
     <col width="14" customWidth="1" min="18" max="18"/>
-    <col width="19" customWidth="1" min="19" max="19"/>
-    <col width="18" customWidth="1" min="20" max="20"/>
+    <col width="18" customWidth="1" min="19" max="19"/>
+    <col width="19" customWidth="1" min="20" max="20"/>
     <col width="14" customWidth="1" min="21" max="21"/>
     <col width="20" customWidth="1" min="22" max="22"/>
     <col width="26" customWidth="1" min="23" max="23"/>
@@ -986,12 +986,12 @@
       </c>
       <c r="S1" s="1" t="inlineStr">
         <is>
+          <t>registration_fee</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
           <t>registration_date</t>
-        </is>
-      </c>
-      <c r="T1" s="1" t="inlineStr">
-        <is>
-          <t>registration_fee</t>
         </is>
       </c>
       <c r="U1" s="1" t="inlineStr">
@@ -13063,7 +13063,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F30"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -13140,25 +13140,23 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
           <t>C:49.0, AS:49.0, AD:49.0</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Mismatch</t>
-        </is>
+      <c r="E3" t="n">
+        <v>0</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Campaign/AdSet/Ad Sales totals must equal Total Sales</t>
+          <t>Campaign/AdSet/Ad Sales totals must equal Attributed Sales (49). 3 unattributed sale(s) correctly excluded from summaries.</t>
         </is>
       </c>
     </row>
@@ -13170,25 +13168,23 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>467948</v>
+        <v>440951</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
           <t>C:440951.0, AS:440951.0, AD:440951.0</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Mismatch</t>
-        </is>
+      <c r="E4" t="n">
+        <v>0</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Campaign/AdSet/Ad Revenue totals must equal Total Revenue</t>
+          <t>Campaign/AdSet/Ad Revenue totals must equal Attributed Revenue (unattributed revenue excluded)</t>
         </is>
       </c>
     </row>
@@ -13283,24 +13279,18 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>&lt;10%</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>5.8% (3)</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
+      <c r="C8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D8" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Warn if &gt; 10%</t>
+          <t>Warn if &gt; 10% unattributed. Current: 5.8% (3 sales)</t>
         </is>
       </c>
     </row>
@@ -13463,7 +13453,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>G. Total Sales</t>
+          <t>INV. Revenue Formula</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -13472,24 +13462,24 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>52</v>
+        <v>0</v>
       </c>
       <c r="D15" t="n">
-        <v>52</v>
+        <v>0</v>
       </c>
       <c r="E15" t="n">
         <v>0</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Golden Report verification for Total Sales</t>
+          <t>Attributed + Unattributed = Total Revenue</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>G. Attributed Sales</t>
+          <t>INV. Spend Formula</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -13498,24 +13488,24 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>49</v>
+        <v>0</v>
       </c>
       <c r="D16" t="n">
-        <v>49</v>
+        <v>0</v>
       </c>
       <c r="E16" t="n">
         <v>0</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Golden Report verification for Attributed Sales</t>
+          <t>Attributed + Unallocated = Raw Meta Spend</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>G. Unattributed Sales</t>
+          <t>INV. Profit Formula</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -13524,353 +13514,15 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D17" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E17" t="n">
         <v>0</v>
       </c>
       <c r="F17" t="inlineStr">
-        <is>
-          <t>Golden Report verification for Unattributed Sales</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>G. Total Revenue</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="C18" t="n">
-        <v>467948</v>
-      </c>
-      <c r="D18" t="n">
-        <v>467948</v>
-      </c>
-      <c r="E18" t="n">
-        <v>0</v>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>Golden Report verification for Total Revenue</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>G. Attributed Revenue</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="C19" t="n">
-        <v>440951</v>
-      </c>
-      <c r="D19" t="n">
-        <v>440951</v>
-      </c>
-      <c r="E19" t="n">
-        <v>0</v>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>Golden Report verification for Attributed Revenue</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>G. Unattributed Revenue</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="C20" t="n">
-        <v>26997</v>
-      </c>
-      <c r="D20" t="n">
-        <v>26997</v>
-      </c>
-      <c r="E20" t="n">
-        <v>0</v>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>Golden Report verification for Unattributed Revenue</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>G. Raw Meta Spend</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="C21" t="n">
-        <v>456047.55</v>
-      </c>
-      <c r="D21" t="n">
-        <v>456047.55</v>
-      </c>
-      <c r="E21" t="n">
-        <v>0</v>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>Golden Report verification for Raw Meta Spend</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>G. Attributed Spend</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="C22" t="n">
-        <v>282120.59</v>
-      </c>
-      <c r="D22" t="n">
-        <v>282120.59</v>
-      </c>
-      <c r="E22" t="n">
-        <v>0</v>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>Golden Report verification for Attributed Spend</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>G. Unallocated Spend</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="C23" t="n">
-        <v>173926.96</v>
-      </c>
-      <c r="D23" t="n">
-        <v>173926.96</v>
-      </c>
-      <c r="E23" t="n">
-        <v>0</v>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>Golden Report verification for Unallocated Spend</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>G. Profit</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="C24" t="n">
-        <v>158830.41</v>
-      </c>
-      <c r="D24" t="n">
-        <v>158830.41</v>
-      </c>
-      <c r="E24" t="n">
-        <v>0</v>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>Golden Report verification for Profit</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>G. ROAS</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="C25" t="n">
-        <v>1.56</v>
-      </c>
-      <c r="D25" t="n">
-        <v>1.56</v>
-      </c>
-      <c r="E25" t="n">
-        <v>0</v>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>Golden Report verification for ROAS</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>G. ROI %</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="C26" t="n">
-        <v>56.3</v>
-      </c>
-      <c r="D26" t="n">
-        <v>56.3</v>
-      </c>
-      <c r="E26" t="n">
-        <v>0</v>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>Golden Report verification for ROI %</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>G. CAC</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="C27" t="n">
-        <v>5757.56</v>
-      </c>
-      <c r="D27" t="n">
-        <v>5757.56</v>
-      </c>
-      <c r="E27" t="n">
-        <v>0</v>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>Golden Report verification for CAC</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>INV. Revenue Formula</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="C28" t="n">
-        <v>0</v>
-      </c>
-      <c r="D28" t="n">
-        <v>0</v>
-      </c>
-      <c r="E28" t="n">
-        <v>0</v>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>Attributed + Unattributed = Total Revenue</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>INV. Spend Formula</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="C29" t="n">
-        <v>0</v>
-      </c>
-      <c r="D29" t="n">
-        <v>0</v>
-      </c>
-      <c r="E29" t="n">
-        <v>0</v>
-      </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>Attributed + Unallocated = Raw Spend</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>INV. Profit Formula</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="C30" t="n">
-        <v>0</v>
-      </c>
-      <c r="D30" t="n">
-        <v>0</v>
-      </c>
-      <c r="E30" t="n">
-        <v>0</v>
-      </c>
-      <c r="F30" t="inlineStr">
         <is>
           <t>Attributed Revenue - Attributed Spend = Profit</t>
         </is>
@@ -13928,8 +13580,8 @@
     <col width="50" customWidth="1" min="16" max="16"/>
     <col width="20" customWidth="1" min="17" max="17"/>
     <col width="14" customWidth="1" min="18" max="18"/>
-    <col width="21" customWidth="1" min="19" max="19"/>
-    <col width="18" customWidth="1" min="20" max="20"/>
+    <col width="18" customWidth="1" min="19" max="19"/>
+    <col width="21" customWidth="1" min="20" max="20"/>
     <col width="14" customWidth="1" min="21" max="21"/>
     <col width="20" customWidth="1" min="22" max="22"/>
     <col width="26" customWidth="1" min="23" max="23"/>
@@ -14030,12 +13682,12 @@
       </c>
       <c r="S1" s="1" t="inlineStr">
         <is>
+          <t>registration_fee</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
           <t>registration_date</t>
-        </is>
-      </c>
-      <c r="T1" s="1" t="inlineStr">
-        <is>
-          <t>registration_fee</t>
         </is>
       </c>
       <c r="U1" s="1" t="inlineStr">
@@ -14149,11 +13801,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="S2" s="3" t="n">
+      <c r="S2" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T2" s="3" t="n">
         <v>46248.79236111111</v>
-      </c>
-      <c r="T2" s="2" t="n">
-        <v>0</v>
       </c>
       <c r="U2" t="inlineStr">
         <is>
@@ -14262,11 +13914,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="S3" s="3" t="n">
+      <c r="S3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T3" s="3" t="n">
         <v>46243.98194444444</v>
-      </c>
-      <c r="T3" s="2" t="n">
-        <v>0</v>
       </c>
       <c r="U3" t="inlineStr">
         <is>
@@ -14375,11 +14027,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="S4" s="3" t="n">
+      <c r="S4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T4" s="3" t="n">
         <v>46245.31944444445</v>
-      </c>
-      <c r="T4" s="2" t="n">
-        <v>0</v>
       </c>
       <c r="U4" t="inlineStr">
         <is>
@@ -14456,10 +14108,10 @@
       <c r="Q5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="S5" s="3" t="n"/>
-      <c r="T5" s="2" t="n">
-        <v/>
-      </c>
+      <c r="S5" s="2" t="n">
+        <v/>
+      </c>
+      <c r="T5" s="3" t="n"/>
       <c r="U5" t="inlineStr">
         <is>
           <t>New</t>
@@ -14567,11 +14219,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="S6" s="3" t="n">
+      <c r="S6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T6" s="3" t="n">
         <v>46243.91458333333</v>
-      </c>
-      <c r="T6" s="2" t="n">
-        <v>0</v>
       </c>
       <c r="U6" t="inlineStr">
         <is>
@@ -14680,11 +14332,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="S7" s="3" t="n">
+      <c r="S7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T7" s="3" t="n">
         <v>46247.64097222222</v>
-      </c>
-      <c r="T7" s="2" t="n">
-        <v>0</v>
       </c>
       <c r="U7" t="inlineStr">
         <is>
@@ -14793,11 +14445,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="S8" s="3" t="n">
+      <c r="S8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T8" s="3" t="n">
         <v>46245.94930555556</v>
-      </c>
-      <c r="T8" s="2" t="n">
-        <v>0</v>
       </c>
       <c r="U8" t="inlineStr">
         <is>
@@ -14901,10 +14553,10 @@
       <c r="Q9" s="2" t="n">
         <v>8275.590714285714</v>
       </c>
-      <c r="S9" s="3" t="n"/>
-      <c r="T9" s="2" t="n">
-        <v/>
-      </c>
+      <c r="S9" s="2" t="n">
+        <v/>
+      </c>
+      <c r="T9" s="3" t="n"/>
       <c r="U9" t="inlineStr">
         <is>
           <t>New</t>
@@ -15012,11 +14664,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="S10" s="3" t="n">
+      <c r="S10" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T10" s="3" t="n">
         <v>46248.52986111111</v>
-      </c>
-      <c r="T10" s="2" t="n">
-        <v>0</v>
       </c>
       <c r="U10" t="inlineStr">
         <is>
@@ -15125,11 +14777,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="S11" s="3" t="n">
+      <c r="S11" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T11" s="3" t="n">
         <v>46249.45555555556</v>
-      </c>
-      <c r="T11" s="2" t="n">
-        <v>0</v>
       </c>
       <c r="U11" t="inlineStr">
         <is>
@@ -15233,10 +14885,10 @@
       <c r="Q12" s="2" t="n">
         <v>8275.590714285714</v>
       </c>
-      <c r="S12" s="3" t="n"/>
-      <c r="T12" s="2" t="n">
-        <v/>
-      </c>
+      <c r="S12" s="2" t="n">
+        <v/>
+      </c>
+      <c r="T12" s="3" t="n"/>
       <c r="U12" t="inlineStr">
         <is>
           <t>New</t>
@@ -15344,11 +14996,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="S13" s="3" t="n">
+      <c r="S13" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T13" s="3" t="n">
         <v>46244.9875</v>
-      </c>
-      <c r="T13" s="2" t="n">
-        <v>0</v>
       </c>
       <c r="U13" t="inlineStr">
         <is>
@@ -15457,11 +15109,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="S14" s="3" t="n">
+      <c r="S14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T14" s="3" t="n">
         <v>46248.38263888889</v>
-      </c>
-      <c r="T14" s="2" t="n">
-        <v>0</v>
       </c>
       <c r="U14" t="inlineStr">
         <is>
@@ -15570,11 +15222,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="S15" s="3" t="n">
+      <c r="S15" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T15" s="3" t="n">
         <v>46247.81805555556</v>
-      </c>
-      <c r="T15" s="2" t="n">
-        <v>0</v>
       </c>
       <c r="U15" t="inlineStr">
         <is>
@@ -15683,11 +15335,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="S16" s="3" t="n">
+      <c r="S16" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T16" s="3" t="n">
         <v>46247.56875</v>
-      </c>
-      <c r="T16" s="2" t="n">
-        <v>0</v>
       </c>
       <c r="U16" t="inlineStr">
         <is>
@@ -15791,10 +15443,10 @@
       <c r="Q17" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="S17" s="3" t="n"/>
-      <c r="T17" s="2" t="n">
-        <v/>
-      </c>
+      <c r="S17" s="2" t="n">
+        <v/>
+      </c>
+      <c r="T17" s="3" t="n"/>
       <c r="U17" t="inlineStr">
         <is>
           <t>New</t>
@@ -15902,11 +15554,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="S18" s="3" t="n">
+      <c r="S18" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T18" s="3" t="n">
         <v>46248.38333333333</v>
-      </c>
-      <c r="T18" s="2" t="n">
-        <v>0</v>
       </c>
       <c r="U18" t="inlineStr">
         <is>
@@ -15983,10 +15635,10 @@
       <c r="Q19" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="S19" s="3" t="n"/>
-      <c r="T19" s="2" t="n">
-        <v/>
-      </c>
+      <c r="S19" s="2" t="n">
+        <v/>
+      </c>
+      <c r="T19" s="3" t="n"/>
       <c r="U19" t="inlineStr">
         <is>
           <t>New</t>
@@ -16094,11 +15746,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="S20" s="3" t="n">
+      <c r="S20" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T20" s="3" t="n">
         <v>46244.35347222222</v>
-      </c>
-      <c r="T20" s="2" t="n">
-        <v>0</v>
       </c>
       <c r="U20" t="inlineStr">
         <is>
@@ -16207,11 +15859,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="S21" s="3" t="n">
+      <c r="S21" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T21" s="3" t="n">
         <v>46243.49444444444</v>
-      </c>
-      <c r="T21" s="2" t="n">
-        <v>0</v>
       </c>
       <c r="U21" t="inlineStr">
         <is>
@@ -16320,11 +15972,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="S22" s="3" t="n">
+      <c r="S22" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T22" s="3" t="n">
         <v>46245.81666666667</v>
-      </c>
-      <c r="T22" s="2" t="n">
-        <v>0</v>
       </c>
       <c r="U22" t="inlineStr">
         <is>
@@ -16428,10 +16080,10 @@
       <c r="Q23" s="2" t="n">
         <v>8275.590714285714</v>
       </c>
-      <c r="S23" s="3" t="n"/>
-      <c r="T23" s="2" t="n">
-        <v/>
-      </c>
+      <c r="S23" s="2" t="n">
+        <v/>
+      </c>
+      <c r="T23" s="3" t="n"/>
       <c r="U23" t="inlineStr">
         <is>
           <t>New</t>
@@ -16539,11 +16191,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="S24" s="3" t="n">
+      <c r="S24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T24" s="3" t="n">
         <v>46247.375</v>
-      </c>
-      <c r="T24" s="2" t="n">
-        <v>0</v>
       </c>
       <c r="U24" t="inlineStr">
         <is>
@@ -16652,11 +16304,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="S25" s="3" t="n">
+      <c r="S25" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T25" s="3" t="n">
         <v>46245.99861111111</v>
-      </c>
-      <c r="T25" s="2" t="n">
-        <v>0</v>
       </c>
       <c r="U25" t="inlineStr">
         <is>
@@ -16765,11 +16417,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="S26" s="3" t="n">
+      <c r="S26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T26" s="3" t="n">
         <v>46247.32152777778</v>
-      </c>
-      <c r="T26" s="2" t="n">
-        <v>0</v>
       </c>
       <c r="U26" t="inlineStr">
         <is>
@@ -16873,10 +16525,10 @@
       <c r="Q27" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="S27" s="3" t="n"/>
-      <c r="T27" s="2" t="n">
-        <v/>
-      </c>
+      <c r="S27" s="2" t="n">
+        <v/>
+      </c>
+      <c r="T27" s="3" t="n"/>
       <c r="U27" t="inlineStr">
         <is>
           <t>New</t>
@@ -16957,11 +16609,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="S28" s="3" t="n">
+      <c r="S28" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T28" s="3" t="n">
         <v>46245.96875</v>
-      </c>
-      <c r="T28" s="2" t="n">
-        <v>0</v>
       </c>
       <c r="U28" t="inlineStr">
         <is>
@@ -17070,11 +16722,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="S29" s="3" t="n">
+      <c r="S29" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T29" s="3" t="n">
         <v>46244.92986111111</v>
-      </c>
-      <c r="T29" s="2" t="n">
-        <v>0</v>
       </c>
       <c r="U29" t="inlineStr">
         <is>
@@ -17183,11 +16835,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="S30" s="3" t="n">
+      <c r="S30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T30" s="3" t="n">
         <v>46247.72847222222</v>
-      </c>
-      <c r="T30" s="2" t="n">
-        <v>0</v>
       </c>
       <c r="U30" t="inlineStr">
         <is>
@@ -17291,10 +16943,10 @@
       <c r="Q31" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="S31" s="3" t="n"/>
-      <c r="T31" s="2" t="n">
-        <v/>
-      </c>
+      <c r="S31" s="2" t="n">
+        <v/>
+      </c>
+      <c r="T31" s="3" t="n"/>
       <c r="U31" t="inlineStr">
         <is>
           <t>New</t>
@@ -17402,11 +17054,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="S32" s="3" t="n">
+      <c r="S32" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T32" s="3" t="n">
         <v>46243.63055555556</v>
-      </c>
-      <c r="T32" s="2" t="n">
-        <v>0</v>
       </c>
       <c r="U32" t="inlineStr">
         <is>
@@ -17515,11 +17167,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="S33" s="3" t="n">
+      <c r="S33" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T33" s="3" t="n">
         <v>46246.63958333333</v>
-      </c>
-      <c r="T33" s="2" t="n">
-        <v>0</v>
       </c>
       <c r="U33" t="inlineStr">
         <is>
@@ -17623,10 +17275,10 @@
       <c r="Q34" s="2" t="n">
         <v>8275.590714285714</v>
       </c>
-      <c r="S34" s="3" t="n"/>
-      <c r="T34" s="2" t="n">
-        <v/>
-      </c>
+      <c r="S34" s="2" t="n">
+        <v/>
+      </c>
+      <c r="T34" s="3" t="n"/>
       <c r="U34" t="inlineStr">
         <is>
           <t>New</t>
@@ -17734,11 +17386,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="S35" s="3" t="n">
+      <c r="S35" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T35" s="3" t="n">
         <v>46248.97569444445</v>
-      </c>
-      <c r="T35" s="2" t="n">
-        <v>0</v>
       </c>
       <c r="U35" t="inlineStr">
         <is>
@@ -17847,11 +17499,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="S36" s="3" t="n">
+      <c r="S36" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T36" s="3" t="n">
         <v>46247.53958333333</v>
-      </c>
-      <c r="T36" s="2" t="n">
-        <v>0</v>
       </c>
       <c r="U36" t="inlineStr">
         <is>
@@ -17960,11 +17612,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="S37" s="3" t="n">
+      <c r="S37" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T37" s="3" t="n">
         <v>46245.68472222222</v>
-      </c>
-      <c r="T37" s="2" t="n">
-        <v>0</v>
       </c>
       <c r="U37" t="inlineStr">
         <is>
@@ -18073,11 +17725,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="S38" s="3" t="n">
+      <c r="S38" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T38" s="3" t="n">
         <v>46247.77708333333</v>
-      </c>
-      <c r="T38" s="2" t="n">
-        <v>0</v>
       </c>
       <c r="U38" t="inlineStr">
         <is>
@@ -18181,10 +17833,10 @@
       <c r="Q39" s="2" t="n">
         <v>8275.590714285714</v>
       </c>
-      <c r="S39" s="3" t="n"/>
-      <c r="T39" s="2" t="n">
-        <v/>
-      </c>
+      <c r="S39" s="2" t="n">
+        <v/>
+      </c>
+      <c r="T39" s="3" t="n"/>
       <c r="U39" t="inlineStr">
         <is>
           <t>New</t>
@@ -18292,11 +17944,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="S40" s="3" t="n">
+      <c r="S40" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T40" s="3" t="n">
         <v>46245.82361111111</v>
-      </c>
-      <c r="T40" s="2" t="n">
-        <v>0</v>
       </c>
       <c r="U40" t="inlineStr">
         <is>
@@ -18405,11 +18057,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="S41" s="3" t="n">
+      <c r="S41" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T41" s="3" t="n">
         <v>46245.41875</v>
-      </c>
-      <c r="T41" s="2" t="n">
-        <v>0</v>
       </c>
       <c r="U41" t="inlineStr">
         <is>
@@ -18513,10 +18165,10 @@
       <c r="Q42" s="2" t="n">
         <v>8275.590714285714</v>
       </c>
-      <c r="S42" s="3" t="n"/>
-      <c r="T42" s="2" t="n">
-        <v/>
-      </c>
+      <c r="S42" s="2" t="n">
+        <v/>
+      </c>
+      <c r="T42" s="3" t="n"/>
       <c r="U42" t="inlineStr">
         <is>
           <t>New</t>
@@ -18619,10 +18271,10 @@
       <c r="Q43" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="S43" s="3" t="n"/>
-      <c r="T43" s="2" t="n">
-        <v/>
-      </c>
+      <c r="S43" s="2" t="n">
+        <v/>
+      </c>
+      <c r="T43" s="3" t="n"/>
       <c r="U43" t="inlineStr">
         <is>
           <t>New</t>
@@ -18730,11 +18382,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="S44" s="3" t="n">
+      <c r="S44" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T44" s="3" t="n">
         <v>46244.30694444444</v>
-      </c>
-      <c r="T44" s="2" t="n">
-        <v>0</v>
       </c>
       <c r="U44" t="inlineStr">
         <is>
@@ -18843,11 +18495,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="S45" s="3" t="n">
+      <c r="S45" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T45" s="3" t="n">
         <v>46248.91944444444</v>
-      </c>
-      <c r="T45" s="2" t="n">
-        <v>0</v>
       </c>
       <c r="U45" t="inlineStr">
         <is>
@@ -18956,11 +18608,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="S46" s="3" t="n">
+      <c r="S46" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T46" s="3" t="n">
         <v>46243.27708333333</v>
-      </c>
-      <c r="T46" s="2" t="n">
-        <v>0</v>
       </c>
       <c r="U46" t="inlineStr">
         <is>
@@ -19064,10 +18716,10 @@
       <c r="Q47" s="2" t="n">
         <v>10080.81</v>
       </c>
-      <c r="S47" s="3" t="n"/>
-      <c r="T47" s="2" t="n">
-        <v/>
-      </c>
+      <c r="S47" s="2" t="n">
+        <v/>
+      </c>
+      <c r="T47" s="3" t="n"/>
       <c r="U47" t="inlineStr">
         <is>
           <t>New</t>
@@ -19175,11 +18827,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="S48" s="3" t="n">
+      <c r="S48" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T48" s="3" t="n">
         <v>46246.52708333333</v>
-      </c>
-      <c r="T48" s="2" t="n">
-        <v>0</v>
       </c>
       <c r="U48" t="inlineStr">
         <is>
@@ -19288,11 +18940,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="S49" s="3" t="n">
+      <c r="S49" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T49" s="3" t="n">
         <v>46243.63333333333</v>
-      </c>
-      <c r="T49" s="2" t="n">
-        <v>0</v>
       </c>
       <c r="U49" t="inlineStr">
         <is>
@@ -19401,11 +19053,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="S50" s="3" t="n">
+      <c r="S50" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T50" s="3" t="n">
         <v>46249.40625</v>
-      </c>
-      <c r="T50" s="2" t="n">
-        <v>0</v>
       </c>
       <c r="U50" t="inlineStr">
         <is>
@@ -19514,11 +19166,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="S51" s="3" t="n">
+      <c r="S51" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T51" s="3" t="n">
         <v>46248.67083333333</v>
-      </c>
-      <c r="T51" s="2" t="n">
-        <v>0</v>
       </c>
       <c r="U51" t="inlineStr">
         <is>
@@ -19623,10 +19275,10 @@
       <c r="Q52" s="2" t="n">
         <v>10080.81</v>
       </c>
-      <c r="S52" s="3" t="n"/>
-      <c r="T52" s="2" t="n">
-        <v/>
-      </c>
+      <c r="S52" s="2" t="n">
+        <v/>
+      </c>
+      <c r="T52" s="3" t="n"/>
       <c r="U52" t="inlineStr">
         <is>
           <t>New</t>
@@ -19729,10 +19381,10 @@
       <c r="Q53" s="2" t="n">
         <v>8275.590714285714</v>
       </c>
-      <c r="S53" s="3" t="n"/>
-      <c r="T53" s="2" t="n">
-        <v/>
-      </c>
+      <c r="S53" s="2" t="n">
+        <v/>
+      </c>
+      <c r="T53" s="3" t="n"/>
       <c r="U53" t="inlineStr">
         <is>
           <t>New</t>
@@ -30067,8 +29719,8 @@
     <col width="9" customWidth="1" min="16" max="16"/>
     <col width="18" customWidth="1" min="17" max="17"/>
     <col width="14" customWidth="1" min="18" max="18"/>
-    <col width="21" customWidth="1" min="19" max="19"/>
-    <col width="18" customWidth="1" min="20" max="20"/>
+    <col width="18" customWidth="1" min="19" max="19"/>
+    <col width="21" customWidth="1" min="20" max="20"/>
     <col width="14" customWidth="1" min="21" max="21"/>
     <col width="20" customWidth="1" min="22" max="22"/>
     <col width="26" customWidth="1" min="23" max="23"/>
@@ -30169,12 +29821,12 @@
       </c>
       <c r="S1" s="1" t="inlineStr">
         <is>
+          <t>registration_fee</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
           <t>registration_date</t>
-        </is>
-      </c>
-      <c r="T1" s="1" t="inlineStr">
-        <is>
-          <t>registration_fee</t>
         </is>
       </c>
       <c r="U1" s="1" t="inlineStr">
@@ -30256,10 +29908,10 @@
       <c r="Q2" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="S2" s="3" t="n"/>
-      <c r="T2" s="2" t="n">
-        <v/>
-      </c>
+      <c r="S2" s="2" t="n">
+        <v/>
+      </c>
+      <c r="T2" s="3" t="n"/>
       <c r="U2" t="inlineStr">
         <is>
           <t>New</t>
@@ -30335,10 +29987,10 @@
       <c r="Q3" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="S3" s="3" t="n"/>
-      <c r="T3" s="2" t="n">
-        <v/>
-      </c>
+      <c r="S3" s="2" t="n">
+        <v/>
+      </c>
+      <c r="T3" s="3" t="n"/>
       <c r="U3" t="inlineStr">
         <is>
           <t>New</t>
@@ -30419,11 +30071,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="S4" s="3" t="n">
+      <c r="S4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T4" s="3" t="n">
         <v>46245.96875</v>
-      </c>
-      <c r="T4" s="2" t="n">
-        <v>0</v>
       </c>
       <c r="U4" t="inlineStr">
         <is>

</xml_diff>